<commit_message>
update scorecard layout and soft stretch ui
</commit_message>
<xml_diff>
--- a/apps/backend/feedback/uat_feedback.xlsx
+++ b/apps/backend/feedback/uat_feedback.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,22 +451,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>9746bded-649d-45e0-95d7-b591a299e813</t>
+          <t>64b3ef23-c949-4078-9a18-87ed5d22f294</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>scorecard</t>
+          <t>dot</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yajas</t>
+          <t>Naren</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Keep Cache and Export button in the same line</t>
+          <t>Compare the PErcentile Ranking of supplier based on the Category</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -476,19 +476,19 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-29T18:57:21.855214</t>
+          <t>2026-08-05T17:46:17.988948</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>705c0fc6-087e-42f1-a52c-9f6ea38bdc86</t>
+          <t>7652d475-cf31-494f-baee-e639433672cd</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>scorecard</t>
+          <t>dot</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -498,43 +498,107 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Check the logics</t>
+          <t>Check the SAZ CanPack data , not making sencse</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>New</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-24T16:26:12.968531</t>
+          <t>2026-08-05T17:44:09.992000</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>9746bded-649d-45e0-95d7-b591a299e813</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>scorecard</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Yajas</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Keep Cache and Export button in the same line</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-07-29T18:57:21.855214</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>705c0fc6-087e-42f1-a52c-9f6ea38bdc86</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>scorecard</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Naren</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Check the logics</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-07-24T16:26:12.968531</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>25d67c15-eb08-4e39-bd46-ac800b8f6216</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
         <is>
           <t>Sarthak</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Improved UI</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>2026-07-23T15:29:19.550357</t>
         </is>

</xml_diff>